<commit_message>
Integration Qwen - success
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42FFCE93-2D2D-41F6-A6A2-6D141F3F37AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98539ED-E7E5-4020-A4EC-9A9AC2D2D607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -61,6 +61,45 @@
   </si>
   <si>
     <t>Completed</t>
+  </si>
+  <si>
+    <t>Synch - Azure Devop XenAnalyticTrans - Local Folder - Github</t>
+  </si>
+  <si>
+    <t>Research API gemini</t>
+  </si>
+  <si>
+    <t>Research API Deepseek</t>
+  </si>
+  <si>
+    <t>Research API Qwen Model</t>
+  </si>
+  <si>
+    <t>Instruction of limitation rules for Gen AI Translation</t>
+  </si>
+  <si>
+    <t>Copy from MSTeams Stanley to words</t>
+  </si>
+  <si>
+    <t>Developing UI</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Integrating UI - Qwen</t>
+  </si>
+  <si>
+    <t>Integrating UI - Claude</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>comparison in budgeting price for all the API key Gen AI</t>
+  </si>
+  <si>
+    <t>Setup key from OpenRouter - get the API key - save in cmd - Qwen</t>
   </si>
 </sst>
 </file>
@@ -157,15 +196,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9D9D9"/>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -179,14 +210,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF9BFFBC"/>
           <bgColor rgb="FF99FFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9DC3E6"/>
-          <bgColor theme="6" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -542,10 +565,10 @@
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.26953125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="54" customWidth="1"/>
-    <col min="4" max="4" width="69.36328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="56.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.81640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -582,34 +605,147 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E3" s="4"/>
+      <c r="A3" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E4" s="4"/>
+      <c r="A4" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E5" s="4"/>
+      <c r="A5" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E6" s="4"/>
+      <c r="A6" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E7" s="4"/>
+      <c r="A7" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E8" s="4"/>
+      <c r="A8" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E9" s="4"/>
+      <c r="A9" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E10" s="4"/>
+      <c r="A10" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E11" s="4"/>
+      <c r="A11" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E12" s="4"/>
+      <c r="A12" s="7">
+        <v>46287</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E13" s="4"/>
@@ -656,40 +792,34 @@
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="E2:E965">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
-      <formula>"Pending on Stanley review"</formula>
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+      <formula>"Pending Review"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Completed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
-      <formula>"On drafting – preparation for training"</formula>
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+      <formula>"Drafting"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
-      <formula>"In progressing"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
-      <formula>"In planning; Not execute in coding"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
+      <formula>"Planning"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
-      <formula>"Complete in pipeline C#"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"Synch in Git"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
-      <formula>"PENDING"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
-      <formula>"Current update"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="8" operator="equal">
+      <formula>"Pending Work"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E27:E965" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusOptions</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E2:E26" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
-      <formula1>"Pending on Stanley review,Completed,On drafting – preparation for training,In progressing,In planning; Not execute in coding,Complete in pipeline C#,Synch in Git,PENDING,Current update"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E26" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
+      <formula1>"Planning, Drafting, In progress, Completed, Synch in Git, Pending Work, Pending Review"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Table - output for different model
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98539ED-E7E5-4020-A4EC-9A9AC2D2D607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6F0A2B-A504-4BEA-B99B-F51A9BE4034B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
   <si>
     <t>Date</t>
   </si>
@@ -100,6 +100,12 @@
   </si>
   <si>
     <t>Setup key from OpenRouter - get the API key - save in cmd - Qwen</t>
+  </si>
+  <si>
+    <t>Insert UI Timing to load model and give output</t>
+  </si>
+  <si>
+    <t>Comparison in ppt</t>
   </si>
 </sst>
 </file>
@@ -748,9 +754,15 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
       <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
       <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
update UI and scenario match with exact project
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6F0A2B-A504-4BEA-B99B-F51A9BE4034B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A09B000-395F-4873-AF29-B017D49BD5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Develop Generative AI Translation - MS Teams Planner</t>
   </si>
   <si>
-    <t>Completed</t>
-  </si>
-  <si>
     <t>Synch - Azure Devop XenAnalyticTrans - Local Folder - Github</t>
   </si>
   <si>
@@ -84,9 +81,6 @@
     <t>Developing UI</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
     <t>Integrating UI - Qwen</t>
   </si>
   <si>
@@ -99,13 +93,28 @@
     <t>comparison in budgeting price for all the API key Gen AI</t>
   </si>
   <si>
-    <t>Setup key from OpenRouter - get the API key - save in cmd - Qwen</t>
-  </si>
-  <si>
     <t>Insert UI Timing to load model and give output</t>
   </si>
   <si>
     <t>Comparison in ppt</t>
+  </si>
+  <si>
+    <t>Synch in Git</t>
+  </si>
+  <si>
+    <t>Pending Work</t>
+  </si>
+  <si>
+    <t>Setup key from OpenRouter - "OPENROUTER_API_KEY"</t>
+  </si>
+  <si>
+    <t>insert in cmd prompt - load in visual studio</t>
+  </si>
+  <si>
+    <t>Setup API key from Claude API faiz - "ANTHROPIC_API_KEY"</t>
+  </si>
+  <si>
+    <t>Setup API key from HuggingFace - "HUGGINGFACE_API_KEY"</t>
   </si>
 </sst>
 </file>
@@ -133,7 +142,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -148,6 +157,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9B9B"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -172,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -198,6 +213,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -263,9 +282,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF9B9B"/>
       <color rgb="FF93FF93"/>
       <color rgb="FF00FF00"/>
-      <color rgb="FFFF9B9B"/>
       <color rgb="FF99FFCC"/>
       <color rgb="FFFFFF99"/>
       <color rgb="FFFFFFAB"/>
@@ -574,7 +593,7 @@
     <col min="1" max="1" width="10.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
     <col min="3" max="3" width="56.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.81640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -607,7 +626,7 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -618,10 +637,10 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -632,10 +651,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -646,10 +665,10 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -660,10 +679,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -674,10 +693,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -688,10 +707,13 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -701,14 +723,14 @@
       <c r="B9" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="E9" s="4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -719,10 +741,10 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -733,10 +755,10 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -747,29 +769,67 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>5</v>
+      </c>
       <c r="C13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="4"/>
+        <v>18</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>5</v>
+      </c>
       <c r="C14" t="s">
-        <v>22</v>
-      </c>
-      <c r="E14" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E15" s="4"/>
+      <c r="A15" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E16" s="4"/>
+      <c r="A16" s="9">
+        <v>46294</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="17" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E17" s="4"/>

</xml_diff>

<commit_message>
Updated UI and model Gen AI
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A09B000-395F-4873-AF29-B017D49BD5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F24AD71-D4D5-4A1F-A999-A842056009B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -115,6 +115,15 @@
   </si>
   <si>
     <t>Setup API key from HuggingFace - "HUGGINGFACE_API_KEY"</t>
+  </si>
+  <si>
+    <t>Mapping key column across different table</t>
+  </si>
+  <si>
+    <t>Generating excel - UI Merge Table</t>
+  </si>
+  <si>
+    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -831,34 +840,56 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E17" s="4"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E18" s="4"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="9">
+        <v>46295</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="9">
+        <v>46295</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E19" s="4"/>
     </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E20" s="4"/>
     </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E21" s="4"/>
     </row>
-    <row r="22" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E22" s="4"/>
     </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E23" s="4"/>
     </row>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E24" s="4"/>
     </row>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E25" s="4"/>
     </row>
-    <row r="26" spans="5:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E26" s="4"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update daily task on XenAnalyticsTrans Project
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F24AD71-D4D5-4A1F-A999-A842056009B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3809C538-D3EB-42A1-999C-5E2670A39811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="37">
   <si>
     <t>Date</t>
   </si>
@@ -124,13 +124,60 @@
   </si>
   <si>
     <t>In progress</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>Generate SCL coding synchronize with scenario</t>
+  </si>
+  <si>
+    <t>when click scenario, SCL language show their respective coding</t>
+  </si>
+  <si>
+    <r>
+      <t>"D:\XenAnalyticTransl\Reference\</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Merge Table UI.xlsx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <t>Refine the whole UI. Take note on the improvement suggested by claude</t>
+  </si>
+  <si>
+    <t>Time consumption for the model to load</t>
+  </si>
+  <si>
+    <t>Stop on Friday. Continue on Monday</t>
+  </si>
+  <si>
+    <t>currently modify. But not have a look at all</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +196,14 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -196,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -226,6 +281,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -601,7 +659,7 @@
   <cols>
     <col min="1" max="1" width="10.36328125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="56.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.6328125" customWidth="1"/>
     <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -851,31 +909,76 @@
         <v>26</v>
       </c>
       <c r="E17" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" s="7">
+        <v>46295</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" s="7">
+        <v>46297</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="9">
-        <v>46295</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E20" s="4"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E22" s="4"/>

</xml_diff>

<commit_message>
Refine SCL translation result and warning handling
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3809C538-D3EB-42A1-999C-5E2670A39811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24712F08-F20B-4AFF-8CFA-AEE0046F4072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="40">
   <si>
     <t>Date</t>
   </si>
@@ -172,12 +172,21 @@
   <si>
     <t>currently modify. But not have a look at all</t>
   </si>
+  <si>
+    <t>Hugging Face - Llama : is very bad very slow</t>
+  </si>
+  <si>
+    <t>thinking to drop out</t>
+  </si>
+  <si>
+    <t>Additon README file</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +210,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -367,6 +382,78 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>373530</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>20544</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>209177</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>76573</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" Requires="we">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Add-in 1" title="Mini Calendar and Date Picker">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F066E9C-F400-0286-6ADB-627A7341F2B5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr>
+              <a:graphicFrameLocks noGrp="1"/>
+            </xdr:cNvGraphicFramePr>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/webextensions/webextension/2010/11">
+              <we:webextensionref xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="2" name="Add-in 1" title="Mini Calendar and Date Picker">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F066E9C-F400-0286-6ADB-627A7341F2B5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -652,12 +739,30 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{4F066E9C-F400-0286-6ADB-627A7341F2B5}">
+  <we:reference id="wa102957665" version="1.3.0.0" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA102957665" version="1.3.0.0" store="WA102957665" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="opt_cal_sys" value="21"/>
+    <we:property name="opt_wn" value="false"/>
+    <we:property name="opt_theme" value="1"/>
+    <we:property name="opt_size" value="0"/>
+    <we:property name="opt_confirm" value="true"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
     <col min="3" max="3" width="61.6328125" customWidth="1"/>
     <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
@@ -981,10 +1086,35 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E22" s="4"/>
+      <c r="A22" s="9">
+        <v>46300</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E23" s="4"/>
+      <c r="A23" s="9">
+        <v>46300</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E24" s="4"/>
@@ -995,8 +1125,12 @@
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E26" s="4"/>
     </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="9"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="E2:E965">
     <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Pending Review"</formula>
@@ -1030,5 +1164,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build control find function in UI
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24712F08-F20B-4AFF-8CFA-AEE0046F4072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782C7DEA-2997-403D-A8F2-A9EBD8ADA9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -180,6 +180,12 @@
   </si>
   <si>
     <t>Additon README file</t>
+  </si>
+  <si>
+    <t>Troubleshoot MCCTrip On Off problem</t>
+  </si>
+  <si>
+    <t>Assign On == 1, Off == 0</t>
   </si>
 </sst>
 </file>
@@ -759,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
@@ -1117,16 +1123,49 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E24" s="4"/>
+      <c r="A24" s="9">
+        <v>46301</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B25" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="E25" s="4"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B26" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B27" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="9"/>
+      <c r="B28" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B29" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Problem in credit for OpenRouter
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782C7DEA-2997-403D-A8F2-A9EBD8ADA9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09B0023-AC04-4F01-8319-C496D308DC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -186,6 +186,15 @@
   </si>
   <si>
     <t>Assign On == 1, Off == 0</t>
+  </si>
+  <si>
+    <t>Add new feature UI Ctrl+F for control find</t>
+  </si>
+  <si>
+    <t>comparison between model</t>
+  </si>
+  <si>
+    <t>OpenRouter model unable to load - credit quota problem</t>
   </si>
 </sst>
 </file>
@@ -765,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
@@ -1140,20 +1149,42 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="9">
+        <v>46302</v>
+      </c>
       <c r="B25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E25" s="4"/>
+      <c r="C25" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="9">
+        <v>46302</v>
+      </c>
       <c r="B26" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="4"/>
+      <c r="C26" t="s">
+        <v>43</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
         <v>29</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -1161,11 +1192,25 @@
       <c r="B28" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="E28" s="4"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="E29" s="4"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E30" s="4"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E31" s="4"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.35">
+      <c r="E33" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -1194,10 +1239,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E27:E965" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E34:E965" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusOptions</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E26" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E33" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
       <formula1>"Planning, Drafting, In progress, Completed, Synch in Git, Pending Work, Pending Review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
add Groq API key in UI
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09B0023-AC04-4F01-8319-C496D308DC2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BCD2A8-ACD7-4548-8AB6-9DD9D4A7D546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -195,6 +195,12 @@
   </si>
   <si>
     <t>OpenRouter model unable to load - credit quota problem</t>
+  </si>
+  <si>
+    <t>Change new key fro OPENROUTER_KEY (PLC_AI_Translator -&gt; XenAITranslator)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All quota for the all model loaded inside the UI is empty. </t>
   </si>
 </sst>
 </file>
@@ -779,7 +785,7 @@
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="61.6328125" customWidth="1"/>
+    <col min="3" max="3" width="71.1796875" customWidth="1"/>
     <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1177,6 +1183,9 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="9">
+        <v>46302</v>
+      </c>
       <c r="B27" s="2" t="s">
         <v>29</v>
       </c>
@@ -1188,17 +1197,32 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="9"/>
+      <c r="A28" s="9">
+        <v>46303</v>
+      </c>
       <c r="B28" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E28" s="4"/>
+      <c r="C28" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="9">
+        <v>46303</v>
+      </c>
       <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E29" s="4"/>
+      <c r="C29" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E30" s="4"/>

</xml_diff>

<commit_message>
Update Groq inside project timeline
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BCD2A8-ACD7-4548-8AB6-9DD9D4A7D546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F02941F-EB39-4C11-A415-1766EC1AB09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="55">
   <si>
     <t>Date</t>
   </si>
@@ -201,6 +201,30 @@
   </si>
   <si>
     <t xml:space="preserve">All quota for the all model loaded inside the UI is empty. </t>
+  </si>
+  <si>
+    <t>Progress as in 9/10/2026</t>
+  </si>
+  <si>
+    <t>Develop Dummy UI to integrate gen AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experimenting gen AI from 4 model - Qwen, Llama, Claude, ChatGPT </t>
+  </si>
+  <si>
+    <t>All 4 model free credit is empty, hence the experimentation is stop</t>
+  </si>
+  <si>
+    <t>Find the solution of free API key source - Groq</t>
+  </si>
+  <si>
+    <t>Insert "GROQ_API_KEY"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seting UI for Groq - Qwen, Llama, GPT </t>
+  </si>
+  <si>
+    <t>Problem in Llama Groq</t>
   </si>
 </sst>
 </file>
@@ -780,7 +804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
@@ -1225,16 +1249,80 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E30" s="4"/>
+      <c r="A30" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E31" s="4"/>
+      <c r="A31" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" t="s">
+        <v>52</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E32" s="4"/>
-    </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.35">
-      <c r="E33" s="4"/>
+      <c r="A32" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C32" t="s">
+        <v>53</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="9">
+        <v>46304</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C33" t="s">
+        <v>54</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C40" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C41" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C42" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C43" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
Update XenAnalyticsTrans Timeline Project - integrate pseudocode
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4C8212-29D5-4780-A5D0-22D2D9BD6327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B6D358-DFEF-4ACC-BFB1-EF9DCCBA52AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Progress" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="62">
   <si>
     <t>Date</t>
   </si>
@@ -233,7 +233,19 @@
     <t>Stop project for a while - focus on XenOptimization</t>
   </si>
   <si>
-    <t>Change the SCL language to psuedocode. Not apply yet inside UI. Just draft in chatgpt</t>
+    <t>= solution is stop using OPEN ROUTER, change to Groq</t>
+  </si>
+  <si>
+    <t>Integrate the pseudocode in UI</t>
+  </si>
+  <si>
+    <t>Refine the README files according to the pseudocode output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove 2 models from Groq Llama due to free-tier access restrictions </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change the SCL language to psuedocode. </t>
   </si>
 </sst>
 </file>
@@ -320,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -352,6 +364,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -443,15 +458,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>373530</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>20544</xdr:rowOff>
+      <xdr:colOff>564030</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>122144</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>209177</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>76573</xdr:rowOff>
+      <xdr:colOff>399677</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>178173</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" Requires="we">
@@ -813,12 +828,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="83.90625" customWidth="1"/>
+    <col min="3" max="3" width="72.453125" customWidth="1"/>
     <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1215,7 +1230,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="9">
         <v>46302</v>
       </c>
@@ -1225,8 +1240,11 @@
       <c r="C27" t="s">
         <v>43</v>
       </c>
+      <c r="D27" s="12" t="s">
+        <v>57</v>
+      </c>
       <c r="E27" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -1299,7 +1317,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="9">
         <v>46304</v>
       </c>
@@ -1309,8 +1327,11 @@
       <c r="C33" t="s">
         <v>51</v>
       </c>
+      <c r="D33" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="E33" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1349,36 +1370,64 @@
         <v>29</v>
       </c>
       <c r="C36" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C40" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="9">
+        <v>46314</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37" t="s">
+        <v>58</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="9">
+        <v>46314</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C47" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C41" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C48" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C42" t="s">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C49" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C43" t="s">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C50" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="E2:E965">
+  <conditionalFormatting sqref="E2:E972">
     <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Pending Review"</formula>
     </cfRule>
@@ -1402,10 +1451,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E37:E965" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E39:E972" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusOptions</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E36" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E38" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
       <formula1>"Planning, Drafting, In progress, Completed, Synch in Git, Pending Work, Pending Review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
save output in db
</commit_message>
<xml_diff>
--- a/Reference/XenAnalyticsTrans Project Timeline.xlsx
+++ b/Reference/XenAnalyticsTrans Project Timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\XenAnalyticTransl\Reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B6D358-DFEF-4ACC-BFB1-EF9DCCBA52AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BF31E92-0B5C-47E9-B620-A3821ED2F40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="66">
   <si>
     <t>Date</t>
   </si>
@@ -246,6 +246,18 @@
   </si>
   <si>
     <t xml:space="preserve">Change the SCL language to psuedocode. </t>
+  </si>
+  <si>
+    <t>completed</t>
+  </si>
+  <si>
+    <t>Refine script LLM Translator - cleaning script</t>
+  </si>
+  <si>
+    <t>Remain only the translator, remove other tab on output</t>
+  </si>
+  <si>
+    <t>Save the output into db, whenever I load the same statement, it just pop out</t>
   </si>
 </sst>
 </file>
@@ -833,8 +845,8 @@
   <cols>
     <col min="1" max="1" width="15.54296875" style="2" customWidth="1"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="72.453125" customWidth="1"/>
-    <col min="4" max="4" width="39.36328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="54.453125" customWidth="1"/>
+    <col min="4" max="4" width="28.36328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1213,7 +1225,7 @@
         <v>42</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -1271,8 +1283,11 @@
       <c r="C29" t="s">
         <v>54</v>
       </c>
+      <c r="D29" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="E29" s="4" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -1403,6 +1418,43 @@
       <c r="E38" s="4" t="s">
         <v>20</v>
       </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="9">
+        <v>46315</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C39" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="9">
+        <v>46315</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C40" t="s">
+        <v>64</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" s="4"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E42" s="4"/>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="C47" t="s">
@@ -1451,10 +1503,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E39:E972" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please select a status from the dropdown list." sqref="E43:E972" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>StatusOptions</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E38" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E42" xr:uid="{8EA7E1BD-2BD4-4FEA-AC5C-45E553151505}">
       <formula1>"Planning, Drafting, In progress, Completed, Synch in Git, Pending Work, Pending Review"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>